<commit_message>
added punch back plate
</commit_message>
<xml_diff>
--- a/Standard_Chart_Template.xlsx
+++ b/Standard_Chart_Template.xlsx
@@ -20,6 +20,8 @@
     <sheet name="Cavityhousingdrilling" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="BoltStandards" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="SpacerBlocksCosting" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="PunchHousingDrilling" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="PunchBackPlate" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -609,6 +611,78 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Diameter</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Thickness</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Diameter</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Thickness</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>